<commit_message>
Cannazone Seattle YTD outputs
</commit_message>
<xml_diff>
--- a/data/cannazone-seattle-ytd.xlsx
+++ b/data/cannazone-seattle-ytd.xlsx
@@ -67,17 +67,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -465,7 +461,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-24T19:15:54.387Z</t>
+          <t>2026-06-24T19:30:54.523Z</t>
         </is>
       </c>
     </row>
@@ -550,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -600,7 +596,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>80974.13000000008</v>
+        <v>80974.13000000005</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>13830</v>
@@ -609,28 +605,12 @@
         <v>523</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>154.8262523900575</v>
+        <v>154.8262523900574</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>2026-06-16</t>
         </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="n">
-        <v>80974.13000000008</v>
-      </c>
-      <c r="C3" s="7" t="n">
-        <v>13830</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>523</v>
       </c>
     </row>
   </sheetData>

</xml_diff>